<commit_message>
Il modello di importazione segue l'elenco del programma
Stesse colonne, stesso ordine, stesse larghezze: chi compila il modello
ritrova quello che vede a video, invece di due disposizioni diverse per
la stessa cosa. Le tendine di Tipo e Stato si agganciano alla posizione
della colonna e non a una lettera scritta a mano, cosi' un riordino non
le lascia indietro.

Rigenerati i due modelli scaricabili dalla pagina del progetto.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Import_template.xlsx
+++ b/docs/Import_template.xlsx
@@ -460,12 +460,12 @@
   <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -481,22 +481,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Model/Description</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Serial number</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <dataValidation sqref="B2:B28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid type" error="Choose Laptop or Tablet." type="list">
       <formula1>"Laptop,Tablet"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid status" error="Choose one of the listed statuses." type="list">
+    <dataValidation sqref="C2:C28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid status" error="Choose one of the listed statuses." type="list">
       <formula1>"Available,Awaiting collection,Faulty - awaiting technician,To be rebuilt,To be checked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Il modello di importazione e' un file esportato vuoto
Erano due formati diversi per la stessa cosa, e chi li usa deve
ricordarsi quale sia quale: prima o poi si sbaglia. Ora il modello ha
esattamente le colonne dell'esportazione - asset tag, tipo, stanza,
note - con la tendina anche sulla stanza. Si esporta, si corregge in
Excel, si reimporta.

Le colonne che il modello non propone piu' restano importabili: chi ha
un foglio suo con modello, seriale o stato lo carica lo stesso, perche'
l'importazione riconosce le colonne dal nome. I file di collaudo le
tengono apposta, per provare proprio quello.

Il collegamento sul desktop punta ad "Avvia Inventario.bat" invece che a
pythonw.exe con argomenti, che su alcune postazioni veniva rifiutato dai
criteri di sicurezza. Se non compare lo stesso, il programma spiega come
farlo a mano - e quella strada non fallisce.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Import_template.xlsx
+++ b/docs/Import_template.xlsx
@@ -457,15 +457,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -481,22 +479,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Room</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Notes</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Model/Description</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Serial number</t>
         </is>
       </c>
     </row>
@@ -512,64 +500,48 @@
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="3" t="n"/>
       <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="3" t="n"/>
       <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -583,64 +555,48 @@
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
       <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -654,77 +610,61 @@
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
       <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
       <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
       <c r="B25" s="3" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
       <c r="B26" s="3" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
       <c r="B27" s="3" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
       <c r="B28" s="3" t="n"/>
       <c r="C28" s="3" t="n"/>
       <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="B2:B28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid type" error="Choose Laptop or Tablet." type="list">
       <formula1>"Laptop,Tablet"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid status" error="Choose one of the listed statuses." type="list">
-      <formula1>"Available,Awaiting collection,Faulty - awaiting technician,To be rebuilt,To be checked"</formula1>
+    <dataValidation sqref="C2:C28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid room" error="Choose one of the configured rooms." type="list">
+      <formula1>"Site Services BAU,Digital Kiosk,Magazzino Disaster Recovery"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -737,7 +677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -794,116 +734,151 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>- Asset Tag and Model are required; the serial number is strongly</t>
+          <t>- The Asset Tag is the only thing required: without it the row is</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  recommended.</t>
+          <t xml:space="preserve">  discarded. Type, room and notes can be left empty.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- The asset tag identifies the device: importing the same asset tag</t>
+          <t>- The template has the same columns as an exported file: you can</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  twice updates the record instead of duplicating it.</t>
+          <t xml:space="preserve">  export, fix things in Excel and import back.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>- Type and Status have dropdowns: use the values offered.</t>
+          <t>- Need other columns? Add them: model, serial number and status are</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>- You can add rows under a separator, or move the separators.</t>
+          <t xml:space="preserve">  recognised by name and imported all the same.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>- Do not change the column names in the first row.</t>
+          <t>- The asset tag identifies the device: importing the same asset tag</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- Rows left empty are simply ignored.</t>
+          <t xml:space="preserve">  twice updates the record instead of duplicating it.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>- Type and Room have dropdowns: use the values offered.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Allowed values</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>- You can leave the room empty: the separators declare it.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Type:  Laptop,  Tablet</t>
+          <t>- You can add rows under a separator, or move the separators.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Status: Available,  Awaiting collection,  Faulty - awaiting technician,  To be rebuilt,  To be checked</t>
+          <t>- Do not change the column names in the first row.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>The dropdowns work in Excel and LibreOffice. Numbers does not import</t>
+          <t>- Rows left empty are simply ignored.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>them: in that case type the values above, they are the same.</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Allowed values</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>iPhones are not imported</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Type:  Laptop,  Tablet</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>They are handled by hand in the program only, and appear neither in</t>
+          <t>Status: Available,  Awaiting collection,  Faulty - awaiting technician,  To be rebuilt,  To be checked</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
+        <is>
+          <t>The dropdowns work in Excel and LibreOffice. Numbers does not import</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>them: in that case type the values above, they are the same.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>iPhones are not imported</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>They are handled by hand in the program only, and appear neither in</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>imports nor in exports. Any you put here will be ignored.</t>
         </is>

</xml_diff>

<commit_message>
Copia e incolla ovunque, tastiera e tasto destro
Le scorciatoie di Tk non sono le stesse su tutti i sistemi ne' con tutte
le disposizioni di tastiera, e in qualche caso non funzionano affatto.
Ora le collega il programma, sulle classi di campo invece che sui
singoli widget - cosi' valgono anche per le finestre costruite dopo - e
sostituendo i collegamenti predefiniti invece di aggiungersi, che
incollerebbe due volte.

Dall'elenco si copia la riga selezionata, incolonnata per Excel, o il
solo identificativo dal tasto destro: e' quello che si incolla in
Elimina +, e chiude il giro nei due sensi.

I percorsi dei file appena esportati erano un'etichetta e non si
potevano copiare: ora sono un campo, e portano il percorso intero.

Documentazione, modelli scaricabili e prove di collaudo aggiornati nelle
due lingue.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Import_template.xlsx
+++ b/docs/Import_template.xlsx
@@ -677,7 +677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -802,83 +802,142 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>- You can add rows under a separator, or move the separators.</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>- Do not change the column names in the first row.</t>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Copy and paste</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>- Rows left empty are simply ignored.</t>
+          <t>- From here you can copy whole columns and paste them into the</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  program: in Delete + you paste asset tags, one per line.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Allowed values</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>- In the program every field accepts Ctrl+C and Ctrl+V, and the</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Type:  Laptop,  Tablet</t>
+          <t xml:space="preserve">  right mouse button opens Copy / Paste.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Status: Available,  Awaiting collection,  Faulty - awaiting technician,  To be rebuilt,  To be checked</t>
+          <t>- From the program's list you copy the selected row with Ctrl+C,</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>The dropdowns work in Excel and LibreOffice. Numbers does not import</t>
+          <t xml:space="preserve">  or just the identifier with the right button: it pastes in</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>them: in that case type the values above, they are the same.</t>
+          <t xml:space="preserve">  here as it is.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>- You can add rows under a separator, or move the separators.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>iPhones are not imported</t>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>- Do not change the column names in the first row.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>- Rows left empty are simply ignored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Allowed values</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Type:  Laptop,  Tablet</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Status: Available,  Awaiting collection,  Faulty - awaiting technician,  To be rebuilt,  To be checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>The dropdowns work in Excel and LibreOffice. Numbers does not import</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>them: in that case type the values above, they are the same.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>iPhones are not imported</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>They are handled by hand in the program only, and appear neither in</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>imports nor in exports. Any you put here will be ignored.</t>
         </is>

</xml_diff>